<commit_message>
Add points for 67uqo1wgdcka1yxqltbiqxn9w_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/67uqo1wgdcka1yxqltbiqxn9w_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/67uqo1wgdcka1yxqltbiqxn9w_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG30"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -819,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -953,14 +953,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -1010,17 +1010,17 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1136,14 +1136,18 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>81</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1151,10 +1155,16 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>81</v>
-      </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+        <v>92.7</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
@@ -1175,10 +1185,10 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF4" t="n">
-        <v>-0.4</v>
+        <v>-0.6000000000000001</v>
       </c>
       <c r="AG4" t="n">
         <v>1</v>
@@ -1189,21 +1199,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.24749085</v>
+        <v>0.04982241999999995</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1221,7 +1231,7 @@
         <v>3</v>
       </c>
       <c r="AS4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT4" t="n">
         <v>0</v>
@@ -1378,11 +1388,11 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
@@ -1504,14 +1514,18 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>81</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1519,10 +1533,16 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>81</v>
-      </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+        <v>92.7</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
@@ -1543,10 +1563,10 @@
         <v>1</v>
       </c>
       <c r="AE6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0.4</v>
+        <v>-0.6000000000000001</v>
       </c>
       <c r="AG6" t="n">
         <v>1</v>
@@ -1557,21 +1577,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.70455117</v>
+        <v>0.72524409</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.31</t>
+          <t>+0.32</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1586,16 +1606,16 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AT6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AU6" t="n">
         <v>3</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>2</v>
       </c>
       <c r="AV6" t="n">
         <v>0</v>
@@ -1742,15 +1762,15 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.13778577</v>
+        <v>0.15252173</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1777,7 +1797,7 @@
         <v>5</v>
       </c>
       <c r="AT7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AU7" t="n">
         <v>0</v>
@@ -1872,14 +1892,18 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>81</v>
-      </c>
-      <c r="O8" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1887,10 +1911,16 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>81</v>
-      </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+        <v>92.7</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
@@ -1911,10 +1941,10 @@
         <v>1</v>
       </c>
       <c r="AE8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF8" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="AG8" t="n">
         <v>1</v>
@@ -1925,21 +1955,21 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.31602856</v>
+        <v>0.2174351</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -1951,10 +1981,10 @@
         <v>1</v>
       </c>
       <c r="AQ8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AR8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AS8" t="n">
         <v>2</v>
@@ -1963,7 +1993,7 @@
         <v>0</v>
       </c>
       <c r="AU8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AV8" t="n">
         <v>1</v>
@@ -1994,7 +2024,7 @@
         <v>0</v>
       </c>
       <c r="BF8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BG8" t="n">
         <v>0</v>
@@ -2055,14 +2085,18 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>81</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2070,10 +2104,16 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>81</v>
-      </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+        <v>92.7</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
@@ -2094,10 +2134,10 @@
         <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF9" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="AG9" t="n">
         <v>1</v>
@@ -2108,21 +2148,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.6520352599999999</v>
+        <v>0.4332538799999999</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+0.26</t>
+          <t>+0.03</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2134,10 +2174,10 @@
         <v>2</v>
       </c>
       <c r="AQ9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AS9" t="n">
         <v>1</v>
@@ -2146,7 +2186,7 @@
         <v>1</v>
       </c>
       <c r="AU9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2177,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BG9" t="n">
         <v>0</v>
@@ -2224,10 +2264,12 @@
           <t>a8pgjuz5yrbxyf1t905gj327d</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -2238,14 +2280,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2253,7 +2295,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2283,7 +2325,7 @@
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -2291,21 +2333,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.8469742099999999</v>
+        <v>0.82513286</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.45</t>
+          <t>+0.42</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2407,10 +2449,12 @@
           <t>cpzl0b545pvfuqec7uaqyhpn8</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2421,14 +2465,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2436,7 +2480,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2466,7 +2510,7 @@
         <v>-0.1</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2474,21 +2518,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.49503431</v>
+        <v>0.43562375</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.10</t>
+          <t>+0.03</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2500,7 +2544,7 @@
         <v>2</v>
       </c>
       <c r="AQ11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR11" t="n">
         <v>1</v>
@@ -2543,7 +2587,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
@@ -2604,14 +2648,18 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>81</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2619,10 +2667,16 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>81</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+        <v>88.09999999999999</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>13.9</v>
+      </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
@@ -2643,10 +2697,10 @@
         <v>1</v>
       </c>
       <c r="AE12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF12" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="AG12" t="n">
         <v>1</v>
@@ -2657,21 +2711,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>1.50704268</v>
+        <v>1.39301515</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+1.11</t>
+          <t>+0.99</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN12" t="n">
         <v>1</v>
@@ -2683,16 +2737,16 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
       </c>
       <c r="AT12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU12" t="n">
         <v>0</v>
@@ -2726,7 +2780,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2780,7 +2834,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L13" t="n">
         <v>2</v>
@@ -2791,14 +2845,18 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>LAM(2), LM</t>
+        </is>
+      </c>
       <c r="P13" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q13" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2806,12 +2864,24 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
+        <v>8.1</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>LM</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
@@ -2830,10 +2900,10 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF13" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG13" t="n">
         <v>2</v>
@@ -2844,21 +2914,21 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0</v>
+        <v>-0.10125564</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.39</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AL13" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AM13" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2873,7 +2943,7 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS13" t="n">
         <v>0</v>
@@ -2882,7 +2952,7 @@
         <v>0</v>
       </c>
       <c r="AU13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV13" t="n">
         <v>0</v>
@@ -2978,14 +3048,18 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>10</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>31</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
       <c r="P14" t="n">
         <v>71</v>
       </c>
       <c r="Q14" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2993,10 +3067,16 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>10</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+        <v>21.7</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -3017,10 +3097,10 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AG14" t="n">
         <v>2</v>
@@ -3031,11 +3111,11 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>-0.225</v>
+        <v>-0.04001580000000005</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.62</t>
+          <t>-0.44</t>
         </is>
       </c>
       <c r="AK14" t="n">
@@ -3045,7 +3125,7 @@
         <v>71</v>
       </c>
       <c r="AM14" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3063,13 +3143,13 @@
         <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AT14" t="n">
         <v>0</v>
       </c>
       <c r="AU14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV14" t="n">
         <v>0</v>
@@ -3165,14 +3245,18 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>LCB(2)</t>
+        </is>
+      </c>
       <c r="P15" t="n">
         <v>80</v>
       </c>
       <c r="Q15" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3180,10 +3264,16 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+        <v>12.7</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>LCB(2)</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
@@ -3204,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG15" t="n">
         <v>2</v>
@@ -3218,21 +3308,21 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0</v>
+        <v>0.02658465999999995</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.39</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AL15" t="n">
         <v>80</v>
       </c>
       <c r="AM15" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3250,7 +3340,7 @@
         <v>0</v>
       </c>
       <c r="AS15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
@@ -3301,37 +3391,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>61g4epojd5f198lv1sje27yh3</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A. Schlager</t>
+          <t>Ali Azaizeh</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>8btyl5lum9zndjh1rxuzdfowl</t>
+          <t>chtopu29kdz63m0vjrmjou1as</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3340,33 +3430,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>88</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>81</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="Q16" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>81</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+        <v>4.7</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -3375,35 +3479,47 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>61g4epojd5f198lv1sje27yh3</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE16" t="n">
         <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>Ali Azaizeh</t>
+        </is>
+      </c>
+      <c r="AI16" t="n">
+        <v>0.17756312</v>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>-0.23</t>
+        </is>
+      </c>
+      <c r="AK16" t="n">
+        <v>19</v>
+      </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="AM16" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3415,10 +3531,10 @@
         <v>0</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS16" t="n">
         <v>0</v>
@@ -3430,7 +3546,7 @@
         <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -3458,7 +3574,7 @@
         <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG16" t="n">
         <v>0</v>
@@ -3472,37 +3588,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>61g4epojd5f198lv1sje27yh3</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>S. Posch</t>
+          <t>Mohammad Al Daoud</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5</t>
+          <t xml:space="preserve"> 25</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1po7tmdv73zfjentt0p20wdlh</t>
+          <t>9eaoefizv7hnz7inuvypc69cl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3511,82 +3627,102 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>87</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>81</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>RB, RWB</t>
+        </is>
+      </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="Q17" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
           <t>RB</t>
         </is>
       </c>
-      <c r="S17" t="n">
-        <v>81</v>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>61g4epojd5f198lv1sje27yh3</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE17" t="n">
         <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>S. Posch</t>
+          <t>Mohammad Al Daoud</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.20397028</v>
+        <v>-0.02473925000000002</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.43</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="AM17" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3598,19 +3734,19 @@
         <v>0</v>
       </c>
       <c r="AQ17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AS17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
         <v>0</v>
@@ -3641,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="BF17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG17" t="n">
         <v>0</v>
@@ -3660,17 +3796,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>P. Mwene</t>
+          <t>A. Schlager</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3680,20 +3816,18 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>7c8ms7bw3fva4xeubax4ep8et</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>2</v>
-      </c>
+          <t>8btyl5lum9zndjh1rxuzdfowl</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
@@ -3704,22 +3838,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3740,38 +3874,26 @@
         </is>
       </c>
       <c r="AD18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE18" t="n">
         <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG18" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>P. Mwene</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>0.17625634</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>-0.22</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>21</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3780,7 +3902,7 @@
         <v>0</v>
       </c>
       <c r="AP18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ18" t="n">
         <v>0</v>
@@ -3798,7 +3920,7 @@
         <v>0</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3826,7 +3948,7 @@
         <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG18" t="n">
         <v>0</v>
@@ -3845,17 +3967,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>X. Schlager</t>
+          <t>S. Posch</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4</t>
+          <t xml:space="preserve"> 5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3865,20 +3987,18 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1s1v1tweyx8wxc9hj2jrnaggl</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>2</v>
-      </c>
+          <t>1po7tmdv73zfjentt0p20wdlh</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -3889,22 +4009,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3925,62 +4045,62 @@
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE19" t="n">
         <v>1</v>
       </c>
       <c r="AF19" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>X. Schlager</t>
+          <t>S. Posch</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.9812843999999999</v>
+        <v>0.2956307399999999</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.59</t>
+          <t>-0.11</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
       </c>
       <c r="AO19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AS19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT19" t="n">
         <v>3</v>
       </c>
       <c r="AU19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4011,7 +4131,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4030,17 +4150,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>P. Lienhart</t>
+          <t>P. Mwene</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4050,18 +4170,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>6o2v57d92t1mejod24gmufcut</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>7c8ms7bw3fva4xeubax4ep8et</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -4072,22 +4194,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4108,7 +4230,7 @@
         </is>
       </c>
       <c r="AD20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE20" t="n">
         <v>1</v>
@@ -4117,29 +4239,29 @@
         <v>-0.2</v>
       </c>
       <c r="AG20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>P. Lienhart</t>
+          <t>P. Mwene</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>1.18839843</v>
+        <v>0.14989698</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.79</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4148,16 +4270,16 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
         <v>0</v>
       </c>
       <c r="AR20" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AS20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT20" t="n">
         <v>0</v>
@@ -4166,7 +4288,7 @@
         <v>0</v>
       </c>
       <c r="AV20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -4194,7 +4316,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4213,17 +4335,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>D. Alaba</t>
+          <t>X. Schlager</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4233,12 +4355,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6w5wyari2p4bh2zzy2x2f6hg5</t>
+          <t>1s1v1tweyx8wxc9hj2jrnaggl</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -4268,7 +4390,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S21" t="n">
@@ -4299,26 +4421,26 @@
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>-0.2</v>
+        <v>-0.05</v>
       </c>
       <c r="AG21" t="n">
         <v>2</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>D. Alaba</t>
+          <t>X. Schlager</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.39105186</v>
+        <v>0.9625650699999999</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>+0.56</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
@@ -4330,28 +4452,28 @@
         <v>0</v>
       </c>
       <c r="AO21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ21" t="n">
         <v>1</v>
       </c>
       <c r="AR21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AS21" t="n">
         <v>3</v>
       </c>
       <c r="AT21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -4379,7 +4501,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -4398,17 +4520,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>R. Schmid</t>
+          <t>P. Lienhart</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 18</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4418,12 +4540,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>b4q9q0qgmtz959rygieg9ln1l</t>
+          <t>6o2v57d92t1mejod24gmufcut</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4440,22 +4562,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4476,68 +4598,68 @@
         </is>
       </c>
       <c r="AD22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE22" t="n">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>R. Schmid</t>
+          <t>P. Lienhart</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.88000841</v>
+        <v>1.49028443</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.49</t>
+          <t>+1.09</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO22" t="n">
         <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AS22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU22" t="n">
         <v>1</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX22" t="n">
         <v>0</v>
@@ -4562,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -4581,17 +4703,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>N. Seiwald</t>
+          <t>D. Alaba</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 8</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4601,18 +4723,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>307whzq643o50rd4g8niobyay</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>6w5wyari2p4bh2zzy2x2f6hg5</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -4623,22 +4747,22 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4659,38 +4783,38 @@
         </is>
       </c>
       <c r="AD23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE23" t="n">
         <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>N. Seiwald</t>
+          <t>D. Alaba</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.33537028</v>
+        <v>0.39105186</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4702,22 +4826,22 @@
         <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AS23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW23" t="n">
         <v>0</v>
@@ -4745,7 +4869,7 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
@@ -4764,17 +4888,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>S. Kalajdžić</t>
+          <t>R. Schmid</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 14</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4784,12 +4908,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>33hs47yxefec8e9ntgqgr49n9</t>
+          <t>b4q9q0qgmtz959rygieg9ln1l</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -4808,22 +4932,22 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
@@ -4844,10 +4968,10 @@
         </is>
       </c>
       <c r="AD24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF24" t="n">
         <v>0</v>
@@ -4857,28 +4981,28 @@
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>S. Kalajdžić</t>
+          <t>R. Schmid</t>
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>0.4168882699999999</v>
+        <v>0.8703887899999999</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>+0.02</t>
+          <t>+0.47</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AL24" t="n">
         <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="AN24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO24" t="n">
         <v>0</v>
@@ -4887,25 +5011,25 @@
         <v>1</v>
       </c>
       <c r="AQ24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT24" t="n">
         <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV24" t="n">
         <v>0</v>
       </c>
       <c r="AW24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX24" t="n">
         <v>0</v>
@@ -4949,17 +5073,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>K. Laimer</t>
+          <t>N. Seiwald</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -4969,12 +5093,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1qthvf5krys0pzk24h8wtr9at</t>
+          <t>307whzq643o50rd4g8niobyay</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -4991,35 +5115,25 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>81</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>LB</t>
-        </is>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S25" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="U25" t="n">
-        <v>22.5</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
@@ -5037,7 +5151,7 @@
         </is>
       </c>
       <c r="AD25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE25" t="n">
         <v>1</v>
@@ -5050,25 +5164,25 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>K. Laimer</t>
+          <t>N. Seiwald</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>0.2799388900000001</v>
+        <v>0.83913659</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>+0.44</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="AL25" t="n">
         <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN25" t="n">
         <v>0</v>
@@ -5083,16 +5197,16 @@
         <v>0</v>
       </c>
       <c r="AR25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV25" t="n">
         <v>0</v>
@@ -5142,17 +5256,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>M. Sabitzer</t>
+          <t>S. Kalajdžić</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 9</t>
+          <t xml:space="preserve"> 14</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -5162,18 +5276,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>8cho2d1nz18i5o0zt6aysd68l</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>33hs47yxefec8e9ntgqgr49n9</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -5184,22 +5300,22 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S26" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
@@ -5220,38 +5336,38 @@
         </is>
       </c>
       <c r="AD26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF26" t="n">
         <v>0</v>
       </c>
       <c r="AG26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>M. Sabitzer</t>
+          <t>S. Kalajdžić</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.6346738699999999</v>
+        <v>0.41682299</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>+0.24</t>
+          <t>+0.01</t>
         </is>
       </c>
       <c r="AK26" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AL26" t="n">
         <v>0</v>
       </c>
       <c r="AM26" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AN26" t="n">
         <v>0</v>
@@ -5263,19 +5379,19 @@
         <v>1</v>
       </c>
       <c r="AQ26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV26" t="n">
         <v>0</v>
@@ -5284,7 +5400,7 @@
         <v>0</v>
       </c>
       <c r="AX26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY26" t="n">
         <v>0</v>
@@ -5306,7 +5422,7 @@
         <v>0</v>
       </c>
       <c r="BF26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BG26" t="n">
         <v>0</v>
@@ -5325,32 +5441,32 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>K. Danso</t>
+          <t>K. Laimer</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3</t>
+          <t xml:space="preserve"> 20</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>4ezld812zytvbokz97jwycgkp</t>
+          <t>1qthvf5krys0pzk24h8wtr9at</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -5359,37 +5475,43 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K27" t="n">
-        <v>58</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2</v>
-      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="N27" t="n">
-        <v>23</v>
-      </c>
-      <c r="O27" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
       <c r="P27" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S27" t="n">
-        <v>23</v>
-      </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
+        <v>58.5</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>43.5</v>
+      </c>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
@@ -5407,38 +5529,38 @@
         </is>
       </c>
       <c r="AD27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF27" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>K. Danso</t>
+          <t>K. Laimer</t>
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.19834416</v>
+        <v>0.42344441</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>-0.20</t>
+          <t>+0.02</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="AL27" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="AM27" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN27" t="n">
         <v>0</v>
@@ -5453,16 +5575,16 @@
         <v>0</v>
       </c>
       <c r="AR27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV27" t="n">
         <v>0</v>
@@ -5512,32 +5634,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M. Arnautović</t>
+          <t>M. Sabitzer</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 9</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>dccxma9p13p00n0gi1cxk1nf9</t>
+          <t>8cho2d1nz18i5o0zt6aysd68l</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -5546,34 +5668,30 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K28" t="n">
-        <v>45</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2</v>
-      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="N28" t="n">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="S28" t="n">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
@@ -5594,7 +5712,7 @@
         </is>
       </c>
       <c r="AD28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE28" t="n">
         <v>1</v>
@@ -5603,29 +5721,29 @@
         <v>0</v>
       </c>
       <c r="AG28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>M. Arnautović</t>
+          <t>M. Sabitzer</t>
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>0.2029539</v>
+        <v>0.73411491</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>+0.33</t>
         </is>
       </c>
       <c r="AK28" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="AL28" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="AM28" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN28" t="n">
         <v>0</v>
@@ -5637,16 +5755,16 @@
         <v>1</v>
       </c>
       <c r="AQ28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU28" t="n">
         <v>1</v>
@@ -5658,7 +5776,7 @@
         <v>0</v>
       </c>
       <c r="AX28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY28" t="n">
         <v>0</v>
@@ -5680,7 +5798,7 @@
         <v>0</v>
       </c>
       <c r="BF28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG28" t="n">
         <v>0</v>
@@ -5699,17 +5817,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>C. Chukwuemeka</t>
+          <t>K. Danso</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5724,7 +5842,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>5ql70wwevaoqpxabylew5f696</t>
+          <t>4ezld812zytvbokz97jwycgkp</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -5745,22 +5863,22 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
         <v>58</v>
       </c>
       <c r="Q29" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S29" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
@@ -5781,7 +5899,7 @@
         </is>
       </c>
       <c r="AD29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE29" t="n">
         <v>0</v>
@@ -5794,25 +5912,25 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>C. Chukwuemeka</t>
+          <t>K. Danso</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>0.08752915</v>
+        <v>0.16943052</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AL29" t="n">
         <v>58</v>
       </c>
       <c r="AM29" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN29" t="n">
         <v>0</v>
@@ -5824,19 +5942,19 @@
         <v>0</v>
       </c>
       <c r="AQ29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT29" t="n">
         <v>0</v>
       </c>
       <c r="AU29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV29" t="n">
         <v>0</v>
@@ -5867,7 +5985,7 @@
         <v>0</v>
       </c>
       <c r="BF29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG29" t="n">
         <v>0</v>
@@ -5886,17 +6004,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>P. Wanner</t>
+          <t>M. Arnautović</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 24</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -5911,7 +6029,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2yc1t7u26zctwjizi283g6q6s</t>
+          <t>dccxma9p13p00n0gi1cxk1nf9</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -5921,7 +6039,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="L30" t="n">
         <v>2</v>
@@ -5932,22 +6050,22 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="Q30" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S30" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
@@ -5968,50 +6086,50 @@
         </is>
       </c>
       <c r="AD30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG30" t="n">
         <v>2</v>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>P. Wanner</t>
+          <t>M. Arnautović</t>
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>-0.02656507</v>
+        <v>1.38234955</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>-0.42</t>
+          <t>+0.98</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AL30" t="n">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="AM30" t="n">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="AN30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO30" t="n">
         <v>0</v>
       </c>
       <c r="AP30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR30" t="n">
         <v>0</v>
@@ -6023,13 +6141,13 @@
         <v>0</v>
       </c>
       <c r="AU30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV30" t="n">
         <v>0</v>
       </c>
       <c r="AW30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX30" t="n">
         <v>0</v>
@@ -6054,9 +6172,570 @@
         <v>0</v>
       </c>
       <c r="BF30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>67uqo1wgdcka1yxqltbiqxn9w</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>C. Chukwuemeka</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 17</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>5ql70wwevaoqpxabylew5f696</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>58</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>44</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>58</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>102</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>44</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>C. Chukwuemeka</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>-0.03981612000000002</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>-0.44</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>58</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>67uqo1wgdcka1yxqltbiqxn9w</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P. Wimmer</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 21</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>aplc9mad75h1k90o3qla9c7l6</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>82</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>20</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>82</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>102</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>20</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>P. Wimmer</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>-0.18876277</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.59</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>82</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>67uqo1wgdcka1yxqltbiqxn9w</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P. Wanner</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 24</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2yc1t7u26zctwjizi283g6q6s</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>58</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>44</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>58</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>102</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>44</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>61g4epojd5f198lv1sje27yh3</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>P. Wanner</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>-0.07857058</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>-0.48</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>28</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>58</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG33" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>